<commit_message>
fix: evaluation > merge + massive bugfix
+ graphiti merge still to be fixed
+ reused existing extract_quintuple function
+ added optional semaphore and atomic facts join in one single string to extract_quintuples()
+ replaced quintuples extraction few shot examples to the expected json format, to facilitate the LLM to generate valid json.
+ removed unused EntitiesExtractor reference inside Relationship's Pydantic model
+ updated vscode debugger config
+ feat: added pickle export format in GraphUtility
</commit_message>
<xml_diff>
--- a/itext2kg_atom/datasets/atom/my_test_datasets/dataset_output.xlsx
+++ b/itext2kg_atom/datasets/atom/my_test_datasets/dataset_output.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mauro\Documents\Andrea\Tesi\itext2kg_atom\datasets\atom\my_test_datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A0603E-82AF-445F-B794-FF4B67493733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8D50A6-C26E-4773-83A3-D8140C3E8EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -40,22 +40,22 @@
     <t>quintuples_g_truth</t>
   </si>
   <si>
+    <t>factoids_extracted_llamacpp_gemma4</t>
+  </si>
+  <si>
+    <t>factoids_prompt_tokenc</t>
+  </si>
+  <si>
+    <t>quintuples_extracted_llamacpp_gemma4</t>
+  </si>
+  <si>
+    <t>quintuples_prompt_tokenc</t>
+  </si>
+  <si>
     <t>quintuples_extracted_from_raw_text_llamacpp_gemma4</t>
   </si>
   <si>
     <t>quintuples_raw_prompt_tokenc</t>
-  </si>
-  <si>
-    <t>quintuples_extracted_llamacpp_gemma4</t>
-  </si>
-  <si>
-    <t>quintuples_prompt_tokenc</t>
-  </si>
-  <si>
-    <t>quintuples_extracted_from_raw_text_llamacpp_gemma4_run2</t>
-  </si>
-  <si>
-    <t>quintuples_extracted_llamacpp_gemma4_run2</t>
   </si>
   <si>
     <t>HONG KONG — Chinese researchers say they have identified a new virus behind an illness that has infected dozens of people across Asia, setting off fears in a region that was struck by a deadly epidemic 17 years ago.</t>
@@ -71,13 +71,13 @@
     <t>[('Chinese Researchers', 'identify', 'New Virus', [], []), ('New Virus', 'cause', 'Illness', [], []), ('new virus', 'infects', 'dozens of people', [], []), ('new virus', 'occurs_in', 'Asia', [], []), ('Outbreak', 'involves', 'New Virus', [], []), ('Outbreak', 'raises', 'Fears', [], []), ('Fears', 'occur_in', 'Asia', [], []), ('Asia', 'experiences', 'Deadly Epidemic', ['2003-01-09'], [])]</t>
   </si>
   <si>
-    <t>[('Chinese researchers', 'identified', 'New virus', [], []), ('New virus', 'is_behind', 'Illness', [], []), ('Illness', 'infected', 'dözens of people', [], []), ('Illness', 'affects', 'Asia', [], []), ('Asia', 'was_struck_by', 'Deadly epidemic', ['2003-01-09'], [])]</t>
-  </si>
-  <si>
-    <t>[('Chinese researchers', 'identify', 'New Virus', [], []), ('New Virus', 'is_cause_of', 'Illness', [], []), ('New Virus', 'infects', 'Dozens of people', [], []), ('New Virus', 'affects_region', 'Asia', [], []), ('Outbreak of the new virus', 'raised', 'Fears', [], []), ('Outbreak of the new virus', 'occurred_in', 'Asia', [], []), ('Asia', 'experienced', 'Deadly Epidemic', ['2003-01-09'], [])]</t>
-  </si>
-  <si>
-    <t>[('Chinese researchers', 'identified', 'New Virus', [], []), ('New Virus', 'is_cause_of', 'Illness', [], []), ('Illness', 'infected', 'Asia', [], []), ('Asia', 'was_struck_by', 'Deadly Epidemic', ['2003-01-09'], ['2003-01-09'])]</t>
+    <t>['Chinese researchers identified a new virus.', 'The new virus is behind an illness.', 'The illness infected dozens of people across Asia.', 'The identification of the virus set off fears in a region.', 'The region was struck by a deadly epidemic on 2003-01-09.']</t>
+  </si>
+  <si>
+    <t>[('Chinese researchers', 'identified', 'new virus', [], []), ('new virus', 'causes', 'illness', [], []), ('The new virus', 'infected', 'dozens of people', ['2020-01-09'], ['2020-01-09']), ('The new virus', 'spread_across', 'Asia', ['2020-01-09'], ['2020-01-09']), ('Outbreak of the New Virus', 'raised_fears_in', 'Asia', [], []), ('Asia', 'experienced', 'Deadly Epidemic', ['2003-01-09'], ['2003-01-09'])]</t>
+  </si>
+  <si>
+    <t>[('Chinese researchers', 'identified', 'new virus', [], []), ('new virus', 'is_behind', 'illness', [], []), ('illness', 'infected_people_in', 'Asia', [], []), ('Asia', 'was_struck_by', 'deadly epidemic', ['2003-01-09'], [])]</t>
   </si>
   <si>
     <t>The spread of a mysterious respiratory virus has prompted the authorities to limit travel in cities in China, including Wuhan, where the disease was first found last month. It has since spread across the nation and to at least 10 other countries.</t>
@@ -93,13 +93,188 @@
     <t>[('Mysterious Respiratory Virus', 'is_found_in', 'Wuhan', ['01-12-2019'], []), ('Authorities', 'impose', 'Travel Limitation', [], []), ('Wuhan', 'is_in', 'China', [], []), ('Travel Limitation', 'is_triggered_by', 'Mysterious Respiratory Virus', [], []), ('Mysterious Respiratory Virus', 'spreads_across', 'China', [], []), ('Mysterious Respiratory Virus', 'spreads_to', 'Other Countries', [], [])]</t>
   </si>
   <si>
-    <t>[('Mysterious Respiratory Virus', 'found_in', 'Wuhan', ['2019-12-23'], []), ('Authorities', 'take_action', 'Limit Travel', [], []), ('Authorities', 'limit_travel_in', 'Cities in China', [], []), ('Cities in China', 'includes', 'Wuhan', [], []), ('Mysterious Respiratory Virus', 'spread_to', 'China', [], []), ('Mysterious Respiratory Virus', 'spread_to', 'At Least 10 Countries', [], [])]</t>
-  </si>
-  <si>
-    <t>[('Mysterious Respiratory Virus', 'found_in', 'Wuhan', ['2019-12-01'], ['2019-12-31']), ('Authorities', 'Authorities limit travel in cities in China', 'limit_travel_in', ['2020-01-23'], []), ('Cities in China', 'Cities in China include Wuhan', 'includes', [], []), ('Limited Travel', 'Limited Travel due to virus spread', 'due_to', [], []), ('Mysterious Respiratory Virus', 'Virus causes travel restrictions', 'causes', [], []), ('Health Officials', 'reported', 'Novel Respiratory Virus', ['2020-01-23'], ['2020-01-23']), ('Novel Respiratory Virus', 'is_named', 'SARS-CoV-2', [], []), ('SARS-CoV-2', 'detected_in', 'Huanan Seafood Wholesale Market', [], []), ('Virus', 'spread_via', 'Respiratory Droplets', [], []), ('Virus', 'caused', 'Concern', [], ['Globally']), ('Mysterious Respiratory Virus', 'spread_to', 'at least 10 other countries', [], [])]</t>
-  </si>
-  <si>
-    <t>[('Authorities', 'take_action', 'Limit Travel', [], []), ('Limit Travel', 'limit_travel_in', 'Cities in China', [], []), ('Mysterious Respiratory Virus', 'causes', 'Authorities', [], []), ('Mysterious Respiratory Virus', 'first_found_in', 'Wuhan', ['2019-12-01'], ['2019-12-31']), ('Mysterious Respiratory Virus', 'spread_across', 'China', [], []), ('Mysterious Respiratory Virus', 'spread_to', 'At Least 10 Other Countries', [], [])]</t>
+    <t>['The spread of a mysterious respiratory virus prompted the authorities to limit travel.', 'The authorities plan to limit travel in cities in China.', 'Wuhan is one of the cities in China where travel will be limited.', 'The mysterious respiratory virus was first found in Wuhan in December 2019.', 'The mysterious respiratory virus has spread across China.', 'The mysterious respiratory virus has spread to at least 10 other countries.']</t>
+  </si>
+  <si>
+    <t>[('Authorities', 'limited', 'Travel', ['2020-01-23'], []), ('Cities in China', 'were_subject_to_restriction_in', 'Travel', ['2020-01-23'], []), ('Wuhan', 'was_restricted_in', 'Travel', ['2020-01-23'], []), ('Mysterious Respiratory Virus', 'caused_restriction_of', 'Travel', [], [])]</t>
+  </si>
+  <si>
+    <t>[('Authorities', 'prompted_to_enact', 'Limit Travel', [], []), ('Limit Travel', 'applies_to', 'Cities in China', [], []), ('Wuhan', 'first_found_in', 'Mysterious Respiratory Virus', ['2019-12-01'], ['2019-12-31']), ('Mysterious Respiratory Virus', 'spread_to', 'China', ['2019-12-01'], ['2020-01-23']), ('Mysterious Respiratory Virus', 'spread_to', 'At least 10 other countries', ['2019-12-01'], ['2020-01-23'])]</t>
+  </si>
+  <si>
+    <t>U.S. stock futures are down sharply this morning on fears about the coronavirus outbreak. More below. (Want this in your inbox each morning? Sign up here.)</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-01-27
+U.S. stock futures are down sharply this morning on fears about the coronavirus outbreak.</t>
+  </si>
+  <si>
+    <t>['U.S. stock futures declined sharply on January 27, 2020.', 'The decline in U.S. stock futures on January 27,2020, was due to fears about the coronavirus outbreak.']</t>
+  </si>
+  <si>
+    <t>[('U.S. stock futures', 'experiences', 'Sharp Decline', ['2020-01-27'], []), ('U.S. stock futures', 'declines_due_to', 'Fears', ['2020-01-27'], []), ('Fears', 'relates_to', 'Coronavirus outbreak', ['2020-01-27'], [])]</t>
+  </si>
+  <si>
+    <t>['U.S. stock futures are down sharply on 2020-01-27.', 'Fears about the coronavirus outbreak caused U.S. stock futures to be down sharply on 2020-01-27.']</t>
+  </si>
+  <si>
+    <t>[('U.S. stock futures', 'declined_sharply', 'Market Decline', ['2020-01-27'], ['2020-01-27']), ('U.S. Stock Futures', 'experienced_decline', 'Decline', ['2020-01-27'], ['2020-01-27']), ('Decline in U.S. Stock Futures', 'caused_by', 'Fears', ['2020-01-27'], ['2020-01-27']), ('Fears', 'concerns', 'Coronavirus Outbreak', ['2020-01-27'], ['2020-01-27'])]</t>
+  </si>
+  <si>
+    <t>[('U.S. stock futures', 'has_status', 'Down Sharply', ['2020-01-27'], ['2020-01-27']), ('U.S. stock futures', 'is_affected_by_fears_about', 'Coronavirus Outbreak', ['2020-01-27'], ['2020-01-27'])]</t>
+  </si>
+  <si>
+    <t>As President Trump’s lawyers open the third day of their defense today, an important question hangs over Washington: Will the Republican-controlled Senate agree to hear testimony from witnesses?.When I flew to China at the beginning of January to teach a three-week college class, the Wuhan coronavirus was barely on anyone’s radar. By the time I got back to New York last Friday, it was front page news around the world, with more than 800 cases in China and 26 deaths; by Monday, the total was at least 80 deaths.. .Hello. On today’s agenda: Apple is scheduled to report earnings today. (Want this in your inbox each morning? Sign up here.)</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-01-28
+As President Trump’s lawyers open the third day of their defense today, an important question hangs over Washington: Will the Republican-controlled Senate agree to hear testimony from witnesses?.When I flew to China at the beginning of January to teach a three-week college class, the Wuhan coronavirus was barely on anyone’s radar. By the time I got back to New York last Friday, it was front page news around the world, with more than 800 cases in China and 26 deaths; by Monday, the total was at least 80 deaths.</t>
+  </si>
+  <si>
+    <t>["President Trump's lawyers began their defense on the third day on January 28, 2020.", 'The Republican-controlled Senate faced the question of whether to hear testimony from witnesses on January 28, 2020.', 'The Wuhan coronavirus was not widely recognized at the beginning of January 2020.', 'By January 24, 2020, the Wuhan coronavirus had become front-page news worldwide.', 'By January 24, 2020, there were over 800 confirmed cases of the Wuhan coronavirus in China.', 'By January 24, 2020, the Wuhan coronavirus had caused 26 deaths in China.', 'By January 27, 2020, the Wuhan coronavirus had caused at least 80 deaths in China.']</t>
+  </si>
+  <si>
+    <t>[("President Trump's lawyers", 'begin_defense', 'Defense', ['2020-01-28'], []), ('Senate', 'considers', 'Hearing Testimony', ['2020-01-28'], []), ('Wuhan coronavirus', 'has_status', 'Not Widely Recognized', ['2020-01-01'], []), ('Wuhan coronavirus', 'has_status', 'Front-page News Worldwide', ['2020-01-24'], []), ('Wuhan coronavirus', 'has_confirmed_cases', 'over 800 confirmed cases', ['24-01-2020'], []), ('Wuhan coronavirus', 'occurs_in', 'China', ['24-01-2020'], []), ('Wuhan coronavirus', 'causes', '26 deaths', [], ['2020-01-24']), ('26 deaths', 'occurs_in', 'China', [], ['2020-01-24']), ('Wuhan coronavirus', 'causes', '80 deaths', [], ['2020-01-27']), ('80 deaths', 'occurs_in', 'China', [], ['2020-01-27'])]</t>
+  </si>
+  <si>
+    <t>["On 2020-01-28, President Trump's lawyers opened the third day of their defense.", 'An important question hangs over Washington regarding whether the Republican-controlled Senate will agree to hear testimony from witnesses.', 'The speaker flew to China at the beginning of January.', 'The speaker traveled to China to teach a three-week college class.', 'When the speaker was in China at the beginning of January, the Wuhan coronavirus was barely on anyone’s radar.', 'When the speaker returned to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'By the time the speaker returned to New York on 2020-01-24, there were more than 800 cases of the Wuhan coronavirus in China.', 'By the time the speaker returned to New York on 2020-01-24, there were 26 deaths from the Wuhan coronavirus in China.', 'By 2020-01-26, the total number of deaths from the Wuhan coronavirus was at least 80.']</t>
+  </si>
+  <si>
+    <t>[("President Trump's lawyers", 'began', 'Defense', ['2020-01-28'], []), ('Republican-controlled Senate', 'faced_question_of', 'Hearing Testimony', ['2020-01-28'], ['2020-01-28']), ('Wuhan coronavirus', 'caused_deaths_in', 'China', [], ['2020-01-24']), ('Wuhan coronavirus', 'caused_deaths_in', 'China', [], ['2020-01-27'])]</t>
+  </si>
+  <si>
+    <t>[('President Trump', 'lawyers open the third day of', 'Defense', ['2020-01-28'], ['2020-01-28']), ('Republican-controlled Senate', 'question hangs over Washington regarding', 'Hearing Testimony', [], []), ('Narrator', 'flew to', 'China', ['2020-01-01'], []), ('Wuhan coronavirus', "was barely on anyone's radar", 'Radar', ['2020-01-01'], []), ('Narrator', 'got back to', 'New York', ['2020-01-24'], []), ('Wuhan coronavirus', 'was', 'Front Page News', ['2020-01-24'], []), ('China', 'had more than 800 cases', 'Wuhan coronavirus', ['2020-01-24'], []), ('China', 'had 26 deaths', 'Wuhan coronavirus', ['2020-01-24'], []), ('China', 'total was at least 80 deaths', 'Wuhan coronavirus', ['2020-01-28'], [])]</t>
+  </si>
+  <si>
+    <t>The World Health Organization declared a global health emergency on Thursday as the coronavirus outbreak spread well beyond China, where it emerged last month.</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-01-30
+The World Health Organization declared a global health emergency on Thursday as the coronavirus outbreak spread well beyond China, where it emerged last month.</t>
+  </si>
+  <si>
+    <t>['The World Health Organization declared a global health emergency on January 30 2020.', 'The coronavirus outbreak spread beyond China on January 30 2020.', 'The coronavirus outbreak emerged in China in December 2019.']</t>
+  </si>
+  <si>
+    <t>[('World Health Organization', 'declares', 'Global Health Emergency', ['30-01-2020'], []), ('coronavirus outbreak', 'spreads_beyond', 'China', ['2020-01-30'], []), ('coronavirus outbreak', 'emerge_in', 'China', ['01-12-2019'], [])]</t>
+  </si>
+  <si>
+    <t>['The World Health Organization declared a global health emergency on 2020-01-30.', 'The coronavirus outbreak spread well beyond China.', 'The coronavirus outbreak emerged in China on December 2019.']</t>
+  </si>
+  <si>
+    <t>[('World Health Organization', 'declared', 'Global Health Emergency', ['2020-01-30'], ['2020-01-30']), ('Coronavirus Outbreak', 'spread_beyond', 'China', [], ['2020-01-30'])]</t>
+  </si>
+  <si>
+    <t>[('World Health Organization', 'declared', 'Global Health Emergency', ['2020-01-30'], ['2020-01-30']), ('Coronavirus Outbreak', 'emerged_in', 'China', ['2019-12-01'], ['2019-12-31']), ('Coronavirus Outbreak', 'spread_beyond', 'China', ['2020-01-30'], ['2020-01-30'])]</t>
+  </si>
+  <si>
+    <t>ANGERS, France — The relentless whir of machines echoing across a cavernous French factory floor this week is an unexpected result of the deadly virus that has nearly paralyzed cities in China and other parts of Asia. The company, Kolmi Hopen, happens to make an item that is suddenly one of the world’s hottest commodities: the medical face mask.</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-02-06
+ANGERS, France — The relentless whir of machines echoing across a cavernous French factory floor this week is an unexpected result of the deadly virus that has nearly paralyzed cities in China and other parts of Asia. The company, Kolmi Hopen, happens to make an item that is suddenly one of the world’s hottest commodities: the medical face mask.</t>
+  </si>
+  <si>
+    <t>['Kolmi Hopen operates a factory in Angers, France on February 3, 2020.', 'Kolmi Hopen produces medical face masks.', 'The demand for medical face masks surged due to the deadly virus outbreak in China and other parts of Asia on February 3, 2020.', 'The virus outbreak nearly paralyzed cities in China and other parts of Asia.', "Kolmi Hopen's factory in France experienced increased production activity due to the high demand for medical face masks on February 3, 2020."]</t>
+  </si>
+  <si>
+    <t>[('Kolmi Hopen', 'operates', 'Factory', ['2020-02-03'], []), ('Factory', 'is_located_in', 'Angers', [], []), ('Angers', 'is_located_in', 'France', [], []), ('Kolmi Hopen', 'produces', 'Medical Face Masks', [], []), ('Virus Outbreak', 'triggers_demand_surge_in', 'Medical Face Masks', ['2020-02-03'], []), ('Virus Outbreak', 'occurs_in', 'China', ['2020-02-03'], []), ('Virus Outbreak', 'occurs_in', 'Asia', ['2020-02-03'], []), ('Virus Outbreak', 'paralyzes', 'Cities', [], []), ('Cities', 'are_located_in', 'China', [], []), ('Cities', 'are_located_in', 'Asia', [], []), ('Kolmi Hopen', 'owns', "Kolmi Hopen's Factory", [], []), ("Kolmi Hopen's Factory", 'is_located_in', 'France', [], []), ("Kolmi Hopen's Factory", 'experiences', 'Increased Production Activity', ['2020-02-03'], []), ('Increased Production Activity', 'is_due_to', 'High Demand for Medical Face Masks', ['2020-02-03'], [])]</t>
+  </si>
+  <si>
+    <t>['The whirring of machines is occurring in a cavernous French factory floor in Angers, France.', 'The whirring of machines is an unexpected result of the deadly virus.', 'The deadly virus nearly paralyzed cities in China.', 'The deadly virus nearly paralyzed cities in other parts of Asia.', 'Kolmi Hopen is the company.', 'Kolmi Hopen makes the medical face mask.', 'The medical face mask is suddenly one of the world’s hottest commodities.']</t>
+  </si>
+  <si>
+    <t>[('Kolmi Hopen', 'operates_factory_in', 'Angers, France', ['2020-02-03'], []), ('Deadly Virus Outbreak', 'occurs_in', 'China', ['2020-02-03'], ['2020-02-03']), ('Deadly Virus Outbreak', 'occurs_in', 'Asia', ['2020-02-03'], ['2020-02-03']), ('Deadly Virus Outbreak', 'causes_demand_surge_for', 'Medical Face Masks', ['2020-02-03'], ['2020-02-03']), ('Medical Face Masks', 'surged', 'Demand Surge', ['2020-02-03'], ['2020-02-03']), ('Virus Outbreak', 'occurred_in', 'China', [], []), ('Virus Outbreak', 'occurred_in', 'Asia', [], []), ('Virus Outbreak', 'nearly_paralyzed', 'Cities', [], []), ("Kolmi Hopen's factory", 'is_located_in', 'France', [], []), ("Kolmi Hopen's factory", 'experienced', 'Increased Production Activity', ['2020-02-03'], ['2020-02-03']), ('Increased Production Activity', 'due_to', 'High Demand for Medical Face Masks', ['2020-02-03'], ['2020-02-03']), ('High Demand for Medical Face Masks', 'relates_to', 'Medical Face Masks', ['2020-02-03'], ['2020-02-03'])]</t>
+  </si>
+  <si>
+    <t>[('Kolmi Hopen', 'manufactures', 'Medical Face Mask', [], []), ('Angers, France', 'is_location_of', 'Kolmi Hopen', [], []), ('Factory Operation', 'is_occurring_at', 'Angers, France', ['2020-02-06'], []), ('Deadly Virus', 'paralyzed', 'China and Asia', [], []), ('Medical Face Mask', 'is_a_hottest_commodity', 'Commodity', [], [])]</t>
+  </si>
+  <si>
+    <t>This year’s edition of Art Basel Hong Kong, one of the most important destinations in the international art market calendar, has been canceled, with organizers citing the ‘‘sudden and widespread outbreak’’ of the coronavirus in China. The fair, held at the Hong Kong Convention and Exhibition Center, and featuring premier galleries from Asia and beyond, was to run March 17  through March 21....Japan already had several confirmed coronavirus cases when a giant cruise ship arrived at the port of Yokohama last week..An alliance between Saudi Arabia and Russia has helped prop up oil prices for the last three years. But the two big oil producers were not in perfect harmony this week, as they have tried to recalibrate production targets to cope with reduced demand from China, whose economy has been crippled by the coronavirus epidemic.</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-02-07This year’s edition of Art Basel Hong Kong, one of the most important destinations in the international art market calendar, has been canceled, with organizers citing the ‘‘sudden and widespread outbreak’’ of the coronavirus in China. The fair, held at the Hong Kong Convention and Exhibition Center, and featuring premier galleries from Asia and beyond, was to run March 17  through March 21.Japan already had several confirmed coronavirus cases when a giant cruise ship arrived at the port of Yokohama last week..An alliance between Saudi Arabia and Russia has helped prop up oil prices for the last three years. But the two big oil producers were not in perfect harmony this week, as they have tried to recalibrate production targets to cope with reduced demand from China, whose economy has been crippled by the coronavirus epidemic.</t>
+  </si>
+  <si>
+    <t>['The 2020 edition of Art Basel Hong Kong was canceled on February 7, 2020.', 'Organizers cited the ‘sudden and widespread outbreak’ of the coronavirus in China as the reason for canceling Art Basel Hong Kong on February 7, 2020.', 'Art Basel Hong Kong was scheduled to be held at the Hong Kong Convention and Exhibition Center from March 17, 2020, to March 21, 2020.', 'Art Basel Hong Kong features premier galleries from Asia and beyond.', 'Japan had several confirmed coronavirus cases by the week of February 3, 2020.', 'A giant cruise ship arrived at the port of Yokohama, Japan, during the week of January 27, 2020.', 'An alliance between Saudi Arabia and Russia has helped prop up oil prices since 2017.', 'Saudi Arabia and Russia were not in perfect harmony during the week of February 3, 2020.', 'Saudi Arabia and Russia tried to recalibrate production targets to cope with reduced demand from China during the week of February 3, 2020.', 'China’s economy was crippled by the coronavirus epidemic on February 7, 2020.']</t>
+  </si>
+  <si>
+    <t>[('Art Basel Hong Kong 2020 edition', 'has_status', 'Canceled', ['2020-02-07'], []), ('Organizers', 'cancel', 'Art Basel Hong Kong', ['2020-02-07'], []), ('Organizers', 'cite', 'Coronavirus Outbreak', ['2020-02-07'], []), ('Coronavirus Outbreak', 'is_located_in', 'China', [], []), ('Art Basel Hong Kong', 'is_held_at', 'Hong Kong Convention and Exhibition Center', ['17-03-2020'], ['21-03-2020']), ('Art Basel Hong Kong', 'features', 'Premier Galleries', [], []), ('Premier Galleries', 'are_from', 'Asia', [], []), ('Japan', 'has_confirmed', 'Confirmed Coronavirus Cases', [], ['2020-02-03']), ('Giant Cruise Ship', 'arrives_at', 'Port of Yokohama', ['2020-01-27'], []), ('Port of Yokohama', 'is_located_in', 'Japan', [], []), ('Saudi Arabia', 'is_allied_with', 'Russia', ['01-01-2017'], []), ('Saudi_Russia_Alliance', 'helps_prop_up', 'Oil Prices', ['01-01-2017'], []), ('Saudi Arabia', 'lack_harmony', 'Russia', ['2020-02-03'], ['2020-02-09']), ('Saudi Arabia', 'recalibrates', 'Production Targets', ['2020-02-03'], []), ('Russia', 'recalibrates', 'Production Targets', ['2020-02-03'], []), ('Production Targets', 'adjusts_for', 'Reduced Demand', ['2020-02-03'], []), ('Reduced Demand', 'originates_from', 'China', ['2020-02-03'], []), ("China's economy", 'is_crippled_by', 'coronavirus epidemic', ['2020-02-07'], [])]</t>
+  </si>
+  <si>
+    <t>['The 2020 edition of Art Basel Hong Kong was canceled.', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China for the cancellation of Art Basel Hong Kong.', 'Art Basel Hong Kong was held at the Hong Kong Convention and Exhibition Center.', 'The fair featured premier galleries from Asia and beyond.', 'The fair was scheduled to run from March 17 through March 21.', 'Japan already had several confirmed coronavirus cases.', 'A giant cruise ship arrived at the port of Yokohama on 2020-02-03 to 2020-02-07.', 'An alliance between Saudi Arabia and Russia helped prop up oil prices for the last three years.', 'Saudi Arabia and Russia were not in perfect harmony this week.', 'Saudi Arabia and Russia tried to recalibrate production targets.', 'Saudi Arabia and Russia recalibrated production targets to cope with reduced demand from China.', "China's economy was crippled by the coronavirus epidemic."]</t>
+  </si>
+  <si>
+    <t>[('Art Basel Hong Kong (2020 edition)', 'has_status', 'Canceled', ['2020-02-07'], ['2020-02-07']), ('Art Basel Hong Kong', 'has_status', 'Canceled', ['2020-02-07'], ['2020-02-07']), ('Coronavirus Outbreak', 'occurs_in', 'China', [], ['2020-02-07']), ('Coronavirus Outbreak', 'caused_cancellation_of', 'Art Basel Hong Kong', [], ['2020-02-07']), ('Art Basel Hong Kong', 'is_scheduled_at', 'Hong Kong Convention and Exhibition Center', ['2020-03-17'], ['2020-03-21']), ('Japan', 'had_confirmed_cases', 'Coronavirus', [], ['2020-02-03']), ('Saudi Arabia', 'forms_alliance_with', 'Russia', ['2017-01-01'], []), ('Saudi Arabia and Russia', 'helped_prop_up', 'Oil Prices', ['2017-01-01'], []), ('Saudi Arabia', 'had_tension_with', 'Russia', ['2020-02-03'], ['2020-02-09']), ("China's Economy", 'was_crippled_by', 'Coronavirus Epidemic', ['2020-02-07'], ['2020-02-07'])]</t>
+  </si>
+  <si>
+    <t>[('Art Basel Hong Kong', 'has_status', 'Canceled', ['2020-03-17'], ['2020-03-21']), ('Art Basel Hong Kong', 'held_at', 'Hong Kong Convention and Exhibition Center', [], []), ('Japan', 'has_confirmed_cases', 'Coronavirus', [], []), ('Giant Cruise Ship', 'arrived_at', 'Port of Yokohama', ['last week'], []), ('Saudi Arabia', 'formed_alliance_with', 'Russia', ['2017-02-07'], ['2020-02-07']), ('Saudi Arabia', 'helped_prop_up', 'Russia', ['2017-02-07'], ['2020-02-07']), ('Saudi Arabia', 'tried_to_recalibrate_production_targets_with', 'Russia', ['2020-02-07'], ['2020-02-07']), ('China', 'crippled_economy_due_to', 'Coronavirus', [], [])]</t>
+  </si>
+  <si>
+    <t>BEIJING — The coronavirus epidemic in China surpassed a grim milestone on Sunday with a death toll that exceeds that of the SARS outbreak 17 years ago, a development that coincided with news that World Health Organization experts might soon be in the country to help stanch the crisis.</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-02-09
+BEIJING — The coronavirus epidemic in China surpassed a grim milestone on Sunday with a death toll that exceeds that of the SARS outbreak 17 years ago, a development that coincided with news that World Health Organization experts might soon be in the country to help stanch the crisis.</t>
+  </si>
+  <si>
+    <t>['The coronavirus epidemic in China surpassed the death toll of the SARS outbreak on February 9, 2020.', 'The SARS outbreak occurred before the coronavirus epidemic milestone in China 17 years before February 9,2020.', 'World Health Organization experts were expected to arrive in China soon to help address the coronavirus crisis on February 9, 2020.']</t>
+  </si>
+  <si>
+    <t>[('Coronavirus Epidemic', 'occurs_in', 'China', [], []), ('Coronavirus Epidemic', 'surpasses', 'SARS Outbreak', ['2020-02-09'], []), ('SARS outbreak', 'occurs_before', 'coronavirus epidemic milestone', [], []), ('coronavirus epidemic milestone', 'is_located_in', 'China', ['2003-02-09'], []), ('World Health Organization experts', 'arrive_in', 'China', ['2020-02-09'], []), ('World Health Organization experts', 'help_address', 'coronavirus crisis', ['2020-02-09'], [])]</t>
+  </si>
+  <si>
+    <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09.', 'The death toll of the coronavirus epidemic in China exceeds the death toll of the SARS outbreak on 2003-02-09.', 'The development coincided with news that World Health Organization experts might soon be in China to help stanch the crisis.']</t>
+  </si>
+  <si>
+    <t>[('Coronavirus epidemic in China', 'surpassed_death_toll_of', 'SARS outbreak', ['2020-02-09'], ['2020-02-09']), ('SARS outbreak', 'occurred_before', 'Coronavirus epidemic milestone in China', [], ['2003-02-09']), ('World Health Organization', 'expected_to_arrive_in', 'China', ['2020-02-09'], ['2020-02-09']), ('World Health Organization', 'expected_to_help_address', 'Coronavirus Crisis', ['2020-02-09'], ['2020-02-09'])]</t>
+  </si>
+  <si>
+    <t>[('Coronavirus epidemic in China', 'reached_milestone', 'Surpassed grim milestone', ['2020-02-09'], ['2020-02-09']), ('Coronavirus epidemic in China', 'death_toll_exceeds', 'SARS outbreak', ['2020-02-09'], ['2020-02-09']), ('World Health Organization experts', 'might_be_in', 'China', [], [])]</t>
+  </si>
+  <si>
+    <t>As many people across China return to work today after an already-extended Lunar New Year break, the country is confronting two bleak statistics:</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-02-10
+As many people across China return to work today after an already-extended Lunar New Year break, the country is confronting two bleak statistics:</t>
+  </si>
+  <si>
+    <t>['People across China returned to work on February 10, 2020, after an extended Lunar New Year break.', 'China faced bleak statistics on February 10, 2020, as people returned to work after the Lunar New Year break.']</t>
+  </si>
+  <si>
+    <t>[('People', 'are_located_in', 'China', [], []), ('People', 'return_to_work', 'Work', ['2020-02-10'], []), ('China', 'faces', 'Bleak Statistics', ['2020-02-10'], []), ('People', 'returns_to_work', 'Work', ['2020-02-10'], []), ('Lunar New Year Break', 'precedes', 'Work', [], [])]</t>
+  </si>
+  <si>
+    <t>['Many people across China are returning to work on 2020-02-10.', 'The Lunar New Year break was extended.', 'China is confronting two bleak statistics.']</t>
+  </si>
+  <si>
+    <t>[('People in China', 'resumed_work', 'Resumed Work', ['2020-02-10'], []), ('Lunar New Year Break', 'ended_before', 'Work', [], ['2020-02-10']), ('China', 'faced_statistics', 'Statistics', ['2020-02-10'], ['2020-02-10']), ('People', 'returned_to_work', 'Returned to Work', ['2020-02-10'], ['2020-02-10']), ('Returning to Work', 'followed_after', 'Lunar New Year Break', ['2020-02-10'], [])]</t>
+  </si>
+  <si>
+    <t>[('People across China', 'returns_to', 'Return to Work', ['2020-02-10'], ['2020-02-10']), ('Lunar New Year Break', 'was_extended', 'Extended', [], []), ('China', 'is_confronting', 'Two Bleak Statistics', ['2020-02-10'], ['2020-02-10'])]</t>
+  </si>
+  <si>
+    <t>NUSA DUA, Indonesia — The family from Shanghai was vacationing in Singapore last month when they learned that the new coronavirus had arrived there from China..When it comes to making decisions that involve risks, we humans can be irrational in quite systematic ways — a fact that the psychologists Amos Tversky and Daniel Kahneman famously demonstrated with the help of a hypothetical situation, eerily apropos of today’s coronavirus epidemic, that has come to be known as the Asian disease problem..A woman sick from the coronavirus was released from a San Diego hospital this week after a labeling error on samples to be tested for the virus led officials to incorrectly indicate that she was not infected, federal authorities said on Tuesday..Chinese health officials said today that the death toll from the coronavirus had passed 1,000. Here are the latest updates and maps of where the virus has reached.</t>
+  </si>
+  <si>
+    <t>Observation date: 2020-02-11
+NUSA DUA, Indonesia — The family from Shanghai was vacationing in Singapore last month when they learned that the new coronavirus had arrived there from China..When it comes to making decisions that involve risks, we humans can be irrational in quite systematic ways — a fact that the psychologists Amos Tversky and Daniel Kahneman famously demonstrated with the help of a hypothetical situation, eerily apropos of today’s coronavirus epidemic, that has come to be known as the Asian disease problem.A woman sick from the coronavirus was released from a San Diego hospital this week after a labeling error on samples to be tested for the virus led officials to incorrectly indicate that she was not infected, federal authorities said on Tuesday.Chinese health officials said today that the death toll from the coronavirus had passed 1,000. Here are the latest updates and maps of where the virus has reached.</t>
+  </si>
+  <si>
+    <t>['A family from Shanghai was vacationing in Singapore in January 2020.', 'The family from Shanghai learned that the new coronavirus had arrived in Singapore from China in January 2020.', 'The new coronavirus arrived in Singapore from China.', 'Humans can be irrational in systematic ways when making decisions that involve risks.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated human irrationality in risk-related decisions.', 'Amos Tversky and Daniel Kahneman used a hypothetical situation called the Asian disease problem.', 'The Asian disease problem is relevant to the coronavirus epidemic of 2020.', 'A woman sick from coronavirus was released from a San Diego hospital during the week of February 10, 2020.', 'The woman was released due to a labeling error on coronavirus test samples.', 'The labeling error led officials to incorrectly indicate that the woman was not infected with coronavirus.', 'Federal authorities reported the San Diego hospital incident on February 11, 2020.', 'Chinese health officials announced on February 11, 2020 that the coronavirus death toll had passed 1,000.']</t>
+  </si>
+  <si>
+    <t>[('Family', 'is_from', 'Shanghai', [], []), ('Family', 'vacations_in', 'Singapore', ['01-01-2020'], ['01-31-2020']), ('Family', 'is_from', 'Shanghai', [], []), ('New Coronavirus', 'arrives_in', 'Singapore', ['01-01-2020'], []), ('New Coronavirus', 'comes_from', 'China', ['01-01-2020'], []), ('Family', 'learns_about', 'New Coronavirus', [], []), ('new coronavirus', 'arrives_in', 'Singapore', [], []), ('new coronavirus', 'originates_from', 'China', [], []), ('Humans', 'exhibit', 'Systematic Irrationality', [], []), ('Humans', 'make', 'Decisions', [], []), ('Decisions', 'involve', 'Risks', [], []), ('Amos Tversky', 'demonstrates', 'Human Irrationality in Risk-Related Decisions', [], []), ('Daniel Kahneman', 'demonstrates', 'Human Irrationality in Risk-Related Decisions', [], []), ('Amos Tversky', 'use', 'Asian disease problem', [], []), ('Daniel Kahneman', 'use', 'Asian disease problem', [], []), ('Asian disease problem', 'is_relevant_to', 'coronavirus epidemic', [], []), ('woman', 'is_sick_with', 'coronavirus', [], []), ('woman', 'is_released_from', 'San Diego hospital', ['2020-02-10'], []), ('woman', 'is_released_due_to', 'Labeling Error', [], []), ('Labeling Error', 'affects', 'Coronavirus Test Samples', [], []), ('Labeling Error', 'leads_to', 'Officials', [], []), ('Officials', 'indicate', 'Woman (not infected with coronavirus)', [], []), ('Federal authorities', 'reports', 'San Diego hospital incident', ['2020-02-11'], []), ('Chinese Health Officials', 'announce', 'Coronavirus Death Toll', ['2020-02-11'], []), ('Coronavirus Death Toll', 'exceed', '1000', ['2020-02-11'], [])]</t>
+  </si>
+  <si>
+    <t>['The family from Shanghai was vacationing in Singapore.', 'The family from Shanghai learned about the new coronavirus arriving in Singapore from China on 2020-01-11.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways.', 'A woman sick from the coronavirus was released from a San Diego hospital.', 'A labeling error on samples led officials to incorrectly indicate that the woman was not infected.', 'Federal authorities said on 2020-02-11 that a woman sick from the coronavirus was released from a San Diego hospital.', 'Chinese health officials said on 2020-02-11 that the death toll from the coronavirus had passed 1,000.']</t>
+  </si>
+  <si>
+    <t>[('New Coronavirus', 'arrived_in', 'Singapore', ['2020-01-01'], ['2020-01-31']), ('New Coronavirus', 'originated_from', 'China', ['2020-01-01'], ['2020-01-31']), ('Family from Shanghai', 'learned_about', 'New Coronavirus', [], []), ('Amos Tversky', 'used', 'Asian disease problem', [], []), ('Daniel Kahneman', 'used', 'Asian disease problem', [], []), ('Asian disease problem', 'is_relevant_to', 'Coronavirus Epidemic', ['2020-01-01'], ['2020-12-31']), ('Woman', 'is_sick_with', 'Coronavirus', ['2020-02-10'], ['2020-02-16']), ('Woman', 'was_treated_at', 'San Diego hospital', ['2020-02-10'], ['2020-02-16']), ('Woman', 'was_released_from', 'Release', ['2020-02-10'], ['2020-02-16']), ('The woman', 'was_released', 'Release', [], []), ('Release', 'due_to', 'Labeling Error', [], []), ('Labeling Error', 'concerns', 'Coronavirus Test Samples', [], []), ('Labeling Error', 'led_to_incorrect_indication', 'Officials', [], []), ('Officials', 'incorrectly_indicated_status_of', 'Woman', [], []), ('Woman', 'was_incorrectly_indicated_as_not_infected_with', 'Coronavirus', [], []), ('Federal authorities', 'reported', 'San Diego hospital incident', ['2020-02-11'], ['2020-02-11']), ('Chinese health officials', 'announced', 'Announcement', ['2020-02-11'], ['2020-02-11']), ('Coronavirus Death Toll', 'passed', '1,000', ['2020-02-11'], ['2020-02-11'])]</t>
+  </si>
+  <si>
+    <t>[('Family from Shanghai', 'was_vacationing_in', 'Singapore', ['2020-01-01'], ['2020-01-31']), ('New Coronavirus', 'arrived_from', 'Singapore', ['2020-01-01'], ['2020-01-31']), ('Humans', 'can_be_irrational_in_systematic_ways', 'Decisions involving risks', [], []), ('Amos Tversky', 'demonstrated', 'Daniel Kahneman', [], []), ('Hypothetical situation', 'was_used_to_demonstrate', 'Coronavirus epidemic', [], []), ('Coronavirus epidemic', 'is_known_as', 'Asian disease problem', [], []), ('Woman', 'was_sick_with', 'Coronavirus', [], []), ('Woman', 'was_released_from', 'San Diego hospital', ['2020-02-11'], ['2020-02-11']), ('Labeling error on samples', 'led_to_incorrect_indication_of', 'Officials', ['2020-02-11'], ['2020-02-11']), ('Chinese health officials', 'reported_passed', 'Coronavirus death toll', ['2020-02-11'], [])]</t>
   </si>
 </sst>
 </file>
@@ -107,7 +282,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -140,7 +315,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -443,18 +618,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
-    <col min="2" max="2" width="3.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="8" max="8" width="34.5703125" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="21.140625" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" customWidth="1"/>
-    <col min="12" max="12" width="57.42578125" customWidth="1"/>
-    <col min="13" max="13" width="17.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+    <col min="10" max="10" width="28.28515625" customWidth="1"/>
+    <col min="12" max="12" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -521,19 +690,19 @@
         <v>16</v>
       </c>
       <c r="I2">
-        <v>762</v>
+        <v>334</v>
       </c>
       <c r="J2" t="s">
         <v>17</v>
       </c>
       <c r="K2">
-        <v>759</v>
+        <v>1719</v>
       </c>
       <c r="L2" t="s">
         <v>18</v>
       </c>
-      <c r="M2" t="s">
-        <v>17</v>
+      <c r="M2">
+        <v>1722</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -562,19 +731,347 @@
         <v>23</v>
       </c>
       <c r="I3">
-        <v>766</v>
+        <v>338</v>
       </c>
       <c r="J3" t="s">
         <v>24</v>
       </c>
       <c r="K3">
-        <v>771</v>
+        <v>1731</v>
       </c>
       <c r="L3" t="s">
         <v>25</v>
       </c>
-      <c r="M3" t="s">
-        <v>24</v>
+      <c r="M3">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>43857</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>307</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4">
+        <v>1711</v>
+      </c>
+      <c r="L4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4">
+        <v>1695</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>43858</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5">
+        <v>398</v>
+      </c>
+      <c r="J5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5">
+        <v>1823</v>
+      </c>
+      <c r="L5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5">
+        <v>1786</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1">
+        <v>43860</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6">
+        <v>316</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K6">
+        <v>1714</v>
+      </c>
+      <c r="L6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6">
+        <v>1704</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>43867</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7">
+        <v>361</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7">
+        <v>1779</v>
+      </c>
+      <c r="L7" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>43868</v>
+      </c>
+      <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8">
+        <v>452</v>
+      </c>
+      <c r="J8" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8">
+        <v>1912</v>
+      </c>
+      <c r="L8" t="s">
+        <v>60</v>
+      </c>
+      <c r="M8">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1">
+        <v>43870</v>
+      </c>
+      <c r="D9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9">
+        <v>347</v>
+      </c>
+      <c r="J9" t="s">
+        <v>66</v>
+      </c>
+      <c r="K9">
+        <v>1743</v>
+      </c>
+      <c r="L9" t="s">
+        <v>67</v>
+      </c>
+      <c r="M9">
+        <v>1735</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1">
+        <v>43871</v>
+      </c>
+      <c r="D10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10">
+        <v>317</v>
+      </c>
+      <c r="J10" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10">
+        <v>1718</v>
+      </c>
+      <c r="L10" t="s">
+        <v>74</v>
+      </c>
+      <c r="M10">
+        <v>1705</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1">
+        <v>43872</v>
+      </c>
+      <c r="D11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I11">
+        <v>463</v>
+      </c>
+      <c r="J11" t="s">
+        <v>80</v>
+      </c>
+      <c r="K11">
+        <v>1889</v>
+      </c>
+      <c r="L11" t="s">
+        <v>81</v>
+      </c>
+      <c r="M11">
+        <v>1851</v>
       </c>
     </row>
   </sheetData>

</xml_diff>